<commit_message>
Sync figure scripts and convergence default with the published analysis
- src/analysis.py: fl_convergence_run now defaults to C.FL_ROUNDS (60) so the
  convergence diagnostic matches the paper's fixed 60 communication rounds
  (was hard-coded 40; elastic net needs ~56 rounds to flatten).
- src/figures.py, regen_figures.py: add the uncorrected-FedAvg overlay
  (hollow orange diamond) and the FL = recalibrated-model remap used in the
  calibration-intercept figures, so regenerated figures match the manuscript.
- outputs/: regenerated figures and tables (raw result CSVs unchanged).

Core analysis code (config, models, flower_fl, calibration, data_utils) is
unchanged and already matched the manuscript.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results.xlsx
+++ b/outputs/results.xlsx
@@ -1177,7 +1177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D165"/>
+  <dimension ref="A1:D245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1861,321 +1861,321 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="C43" t="n">
-        <v>0.6931471805599455</v>
+        <v>0.2017171839256574</v>
       </c>
       <c r="D43" t="n">
-        <v>0.5</v>
+        <v>0.8223571724258368</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="C44" t="n">
-        <v>0.2031895377025221</v>
+        <v>0.2017171892088401</v>
       </c>
       <c r="D44" t="n">
-        <v>0.8212123798334194</v>
+        <v>0.8223568861260985</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="C45" t="n">
-        <v>0.2029479423056985</v>
+        <v>0.2017171938492245</v>
       </c>
       <c r="D45" t="n">
-        <v>0.8214290256160595</v>
+        <v>0.822356812242295</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="C46" t="n">
-        <v>0.2023796361669025</v>
+        <v>0.2017171979051451</v>
       </c>
       <c r="D46" t="n">
-        <v>0.8212593791678835</v>
+        <v>0.8223570985420333</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="C47" t="n">
-        <v>0.2028071139030353</v>
+        <v>0.2017172014364665</v>
       </c>
       <c r="D47" t="n">
-        <v>0.8214565196264151</v>
+        <v>0.8223570431291808</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C48" t="n">
-        <v>0.2028080084473869</v>
+        <v>0.2017172045014542</v>
       </c>
       <c r="D48" t="n">
-        <v>0.8218127411492305</v>
+        <v>0.8223572463096402</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C49" t="n">
-        <v>0.2028075591326614</v>
+        <v>0.201717207154957</v>
       </c>
       <c r="D49" t="n">
-        <v>0.8210722869066198</v>
+        <v>0.8223570154227546</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="C50" t="n">
-        <v>0.2024108534426932</v>
+        <v>0.2017172094474561</v>
       </c>
       <c r="D50" t="n">
-        <v>0.8218061100778719</v>
+        <v>0.8223570154227543</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="C51" t="n">
-        <v>0.2021637441662976</v>
+        <v>0.2017172114246749</v>
       </c>
       <c r="D51" t="n">
-        <v>0.8222948514376343</v>
+        <v>0.8223569877163281</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="C52" t="n">
-        <v>0.2027029949365832</v>
+        <v>0.2017172131275426</v>
       </c>
       <c r="D52" t="n">
-        <v>0.8213062584411668</v>
+        <v>0.8223571539548858</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="C53" t="n">
-        <v>0.2024401715169039</v>
+        <v>0.2017172145923732</v>
       </c>
       <c r="D53" t="n">
-        <v>0.8218856182858497</v>
+        <v>0.8223571077775087</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="C54" t="n">
-        <v>0.2023875858554224</v>
+        <v>0.2017172158511664</v>
       </c>
       <c r="D54" t="n">
-        <v>0.8218930528435712</v>
+        <v>0.8223569692453774</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="C55" t="n">
-        <v>0.2024996057808019</v>
+        <v>0.2017172169319697</v>
       </c>
       <c r="D55" t="n">
-        <v>0.8214612481898352</v>
+        <v>0.8223569784808527</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="C56" t="n">
-        <v>0.2024555359184279</v>
+        <v>0.2017172178592626</v>
       </c>
       <c r="D56" t="n">
-        <v>0.8213035432113903</v>
+        <v>0.8223569784808529</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="C57" t="n">
-        <v>0.2022386122930053</v>
+        <v>0.2017172186543379</v>
       </c>
       <c r="D57" t="n">
-        <v>0.8223049088703777</v>
+        <v>0.8223570338937054</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="C58" t="n">
-        <v>0.2032004836363223</v>
+        <v>0.2017172193356657</v>
       </c>
       <c r="D58" t="n">
-        <v>0.820879607182721</v>
+        <v>0.8223570893065579</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="C59" t="n">
-        <v>0.2026563992253713</v>
+        <v>0.2017172199192311</v>
       </c>
       <c r="D59" t="n">
-        <v>0.8211708571358858</v>
+        <v>0.8223570800710825</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="C60" t="n">
-        <v>0.2023767569354137</v>
+        <v>0.2017172204188427</v>
       </c>
       <c r="D60" t="n">
-        <v>0.8216891612525001</v>
+        <v>0.8223570338937053</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="C61" t="n">
-        <v>0.2022813241647623</v>
+        <v>0.201717220846411</v>
       </c>
       <c r="D61" t="n">
-        <v>0.8219565559726285</v>
+        <v>0.8223570523646563</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>l1</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="C62" t="n">
-        <v>0.2027652237764222</v>
+        <v>0.2017172212121954</v>
       </c>
       <c r="D62" t="n">
-        <v>0.8210783823204038</v>
+        <v>0.8223570616001317</v>
       </c>
     </row>
     <row r="63">
@@ -2185,13 +2185,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>0.2023424593662917</v>
+        <v>0.6931471805599455</v>
       </c>
       <c r="D63" t="n">
-        <v>0.8220959192968692</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="64">
@@ -2201,13 +2201,13 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="C64" t="n">
-        <v>0.2027976186358</v>
+        <v>0.2032318219434939</v>
       </c>
       <c r="D64" t="n">
-        <v>0.8221250018089988</v>
+        <v>0.8219733830088622</v>
       </c>
     </row>
     <row r="65">
@@ -2217,13 +2217,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="C65" t="n">
-        <v>0.2026523676810392</v>
+        <v>0.2026819457521869</v>
       </c>
       <c r="D65" t="n">
-        <v>0.821328377404822</v>
+        <v>0.8219925743268061</v>
       </c>
     </row>
     <row r="66">
@@ -2233,13 +2233,13 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="C66" t="n">
-        <v>0.2025969150818789</v>
+        <v>0.2025301338503157</v>
       </c>
       <c r="D66" t="n">
-        <v>0.8211006952290429</v>
+        <v>0.821627348215446</v>
       </c>
     </row>
     <row r="67">
@@ -2249,13 +2249,13 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="C67" t="n">
-        <v>0.2025495167943198</v>
+        <v>0.2027484767475014</v>
       </c>
       <c r="D67" t="n">
-        <v>0.8215778091252389</v>
+        <v>0.8215045440986517</v>
       </c>
     </row>
     <row r="68">
@@ -2265,13 +2265,13 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="C68" t="n">
-        <v>0.2026079658331789</v>
+        <v>0.2024194669433853</v>
       </c>
       <c r="D68" t="n">
-        <v>0.8215713719988642</v>
+        <v>0.821048690266896</v>
       </c>
     </row>
     <row r="69">
@@ -2281,13 +2281,13 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="C69" t="n">
-        <v>0.2022904448749761</v>
+        <v>0.2026115926571845</v>
       </c>
       <c r="D69" t="n">
-        <v>0.8221259345920171</v>
+        <v>0.8221034000319677</v>
       </c>
     </row>
     <row r="70">
@@ -2297,13 +2297,13 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="C70" t="n">
-        <v>0.2023449207918901</v>
+        <v>0.2027580654313657</v>
       </c>
       <c r="D70" t="n">
-        <v>0.8217905852436739</v>
+        <v>0.821600999404044</v>
       </c>
     </row>
     <row r="71">
@@ -2313,13 +2313,13 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="C71" t="n">
-        <v>0.2026369290897763</v>
+        <v>0.2027383782754792</v>
       </c>
       <c r="D71" t="n">
-        <v>0.8213874290347223</v>
+        <v>0.8210055328902108</v>
       </c>
     </row>
     <row r="72">
@@ -2329,13 +2329,13 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C72" t="n">
-        <v>0.202782646102634</v>
+        <v>0.2025262874385713</v>
       </c>
       <c r="D72" t="n">
-        <v>0.8209448373456842</v>
+        <v>0.8215300617172652</v>
       </c>
     </row>
     <row r="73">
@@ -2345,13 +2345,13 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C73" t="n">
-        <v>0.2023734369376562</v>
+        <v>0.2028833507626904</v>
       </c>
       <c r="D73" t="n">
-        <v>0.8216402224681958</v>
+        <v>0.8209037579509709</v>
       </c>
     </row>
     <row r="74">
@@ -2361,13 +2361,13 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="C74" t="n">
-        <v>0.2025318077260245</v>
+        <v>0.2022711426438486</v>
       </c>
       <c r="D74" t="n">
-        <v>0.8211349773138396</v>
+        <v>0.8218668795062021</v>
       </c>
     </row>
     <row r="75">
@@ -2377,13 +2377,13 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C75" t="n">
-        <v>0.2025245128863345</v>
+        <v>0.2029295214231868</v>
       </c>
       <c r="D75" t="n">
-        <v>0.8219424349306959</v>
+        <v>0.8203562235546202</v>
       </c>
     </row>
     <row r="76">
@@ -2393,13 +2393,13 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="C76" t="n">
-        <v>0.2022690872644851</v>
+        <v>0.2024951438614885</v>
       </c>
       <c r="D76" t="n">
-        <v>0.8220999459641566</v>
+        <v>0.8217725853020603</v>
       </c>
     </row>
     <row r="77">
@@ -2409,13 +2409,13 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="C77" t="n">
-        <v>0.2025882850641921</v>
+        <v>0.2022502389258328</v>
       </c>
       <c r="D77" t="n">
-        <v>0.8216383661376343</v>
+        <v>0.8215756295530374</v>
       </c>
     </row>
     <row r="78">
@@ -2425,13 +2425,13 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="C78" t="n">
-        <v>0.2025698126747558</v>
+        <v>0.2025192819729224</v>
       </c>
       <c r="D78" t="n">
-        <v>0.8219059640382224</v>
+        <v>0.8215595875322154</v>
       </c>
     </row>
     <row r="79">
@@ -2441,13 +2441,13 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="C79" t="n">
-        <v>0.2028235083674469</v>
+        <v>0.2029848934003392</v>
       </c>
       <c r="D79" t="n">
-        <v>0.8217718834059278</v>
+        <v>0.820089696969182</v>
       </c>
     </row>
     <row r="80">
@@ -2457,13 +2457,13 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="C80" t="n">
-        <v>0.2024830061172982</v>
+        <v>0.2025684866523673</v>
       </c>
       <c r="D80" t="n">
-        <v>0.8217830583311982</v>
+        <v>0.8219191707680874</v>
       </c>
     </row>
     <row r="81">
@@ -2473,13 +2473,13 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C81" t="n">
-        <v>0.2029751745046938</v>
+        <v>0.2024785391764745</v>
       </c>
       <c r="D81" t="n">
-        <v>0.8217229261506726</v>
+        <v>0.8213125570354101</v>
       </c>
     </row>
     <row r="82">
@@ -2489,13 +2489,13 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="C82" t="n">
-        <v>0.2025469146686529</v>
+        <v>0.2023357463318786</v>
       </c>
       <c r="D82" t="n">
-        <v>0.8210521905120839</v>
+        <v>0.8221847553350315</v>
       </c>
     </row>
     <row r="83">
@@ -2505,653 +2505,653 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C83" t="n">
-        <v>0.2024485277561125</v>
+        <v>0.2024146318278888</v>
       </c>
       <c r="D83" t="n">
-        <v>0.8215813832542304</v>
+        <v>0.8217344520240093</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="C84" t="n">
-        <v>0.6931471805599455</v>
+        <v>0.202409080086889</v>
       </c>
       <c r="D84" t="n">
-        <v>0.5</v>
+        <v>0.8220151827706591</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="C85" t="n">
-        <v>0.3906801576744426</v>
+        <v>0.2024516218343095</v>
       </c>
       <c r="D85" t="n">
-        <v>0.8088056637919926</v>
+        <v>0.8217540312319213</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="C86" t="n">
-        <v>0.2545362417751943</v>
+        <v>0.2024571431935578</v>
       </c>
       <c r="D86" t="n">
-        <v>0.811068835517097</v>
+        <v>0.8220286111519344</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C87" t="n">
-        <v>0.210901485567246</v>
+        <v>0.2027360381575453</v>
       </c>
       <c r="D87" t="n">
-        <v>0.8145665686557994</v>
+        <v>0.8213144133659717</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="C88" t="n">
-        <v>0.2064513030933844</v>
+        <v>0.2024902486489493</v>
       </c>
       <c r="D88" t="n">
-        <v>0.8174073639562058</v>
+        <v>0.821194204417773</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="C89" t="n">
-        <v>0.2040834515376947</v>
+        <v>0.2025218981985903</v>
       </c>
       <c r="D89" t="n">
-        <v>0.8196404649733098</v>
+        <v>0.8217713662193036</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="C90" t="n">
-        <v>0.2029993016438274</v>
+        <v>0.2024879197285297</v>
       </c>
       <c r="D90" t="n">
-        <v>0.8208928785609141</v>
+        <v>0.8216043888235269</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="C91" t="n">
-        <v>0.2024152001412173</v>
+        <v>0.2026196541976325</v>
       </c>
       <c r="D91" t="n">
-        <v>0.8215591257584437</v>
+        <v>0.8219065458731744</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C92" t="n">
-        <v>0.2021481215593203</v>
+        <v>0.2023049165173431</v>
       </c>
       <c r="D92" t="n">
-        <v>0.8217782004711218</v>
+        <v>0.8220767556853517</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="C93" t="n">
-        <v>0.2019847968926103</v>
+        <v>0.2027716677022941</v>
       </c>
       <c r="D93" t="n">
-        <v>0.8219988452146232</v>
+        <v>0.8223520559724485</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C94" t="n">
-        <v>0.2018962511558601</v>
+        <v>0.2025474307203889</v>
       </c>
       <c r="D94" t="n">
-        <v>0.8220793600894231</v>
+        <v>0.8217961080579809</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="C95" t="n">
-        <v>0.2018349437256716</v>
+        <v>0.2024227204173875</v>
       </c>
       <c r="D95" t="n">
-        <v>0.8221670139867304</v>
+        <v>0.8211275150496921</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="C96" t="n">
-        <v>0.2017970290297426</v>
+        <v>0.2028988649539648</v>
       </c>
       <c r="D96" t="n">
-        <v>0.8222180769303837</v>
+        <v>0.8217348214430266</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C97" t="n">
-        <v>0.2017706927938434</v>
+        <v>0.202338129023709</v>
       </c>
       <c r="D97" t="n">
-        <v>0.8222581127163733</v>
+        <v>0.8222185941170077</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="C98" t="n">
-        <v>0.2017534903193746</v>
+        <v>0.202616862129242</v>
       </c>
       <c r="D98" t="n">
-        <v>0.822279280426059</v>
+        <v>0.8208020107181572</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="C99" t="n">
-        <v>0.2017416439753799</v>
+        <v>0.2021709966812067</v>
       </c>
       <c r="D99" t="n">
-        <v>0.8223010022642707</v>
+        <v>0.8218143111800538</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="C100" t="n">
-        <v>0.2017337112271332</v>
+        <v>0.2027134378957668</v>
       </c>
       <c r="D100" t="n">
-        <v>0.8223150771288262</v>
+        <v>0.8216807107924815</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="C101" t="n">
-        <v>0.2017282807899307</v>
+        <v>0.202336058073892</v>
       </c>
       <c r="D101" t="n">
-        <v>0.8223243033687809</v>
+        <v>0.8215417261227335</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="C102" t="n">
-        <v>0.2017246082583725</v>
+        <v>0.202366343008331</v>
       </c>
       <c r="D102" t="n">
-        <v>0.8223317379265023</v>
+        <v>0.8217861799218935</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="C103" t="n">
-        <v>0.2017221083889447</v>
+        <v>0.2026440761954625</v>
       </c>
       <c r="D103" t="n">
-        <v>0.8223356907099862</v>
+        <v>0.8220987361168755</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="C104" t="n">
-        <v>0.2017204173772831</v>
+        <v>0.2023381265280376</v>
       </c>
       <c r="D104" t="n">
-        <v>0.8223408441052764</v>
+        <v>0.8218662053164957</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="C105" t="n">
-        <v>0.201719273840277</v>
+        <v>0.202679972126314</v>
       </c>
       <c r="D105" t="n">
-        <v>0.8223436701607579</v>
+        <v>0.8219152364555542</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="C106" t="n">
-        <v>0.201718505792623</v>
+        <v>0.2024541433119072</v>
       </c>
       <c r="D106" t="n">
-        <v>0.8223464500388623</v>
+        <v>0.8217497829132233</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="C107" t="n">
-        <v>0.2017179930012444</v>
+        <v>0.202890317716324</v>
       </c>
       <c r="D107" t="n">
-        <v>0.822348823556048</v>
+        <v>0.8217984261623139</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="C108" t="n">
-        <v>0.2017176543508925</v>
+        <v>0.20255363294327</v>
       </c>
       <c r="D108" t="n">
-        <v>0.8223504674706743</v>
+        <v>0.8214651178540405</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="C109" t="n">
-        <v>0.2017174337751697</v>
+        <v>0.2024748827250314</v>
       </c>
       <c r="D109" t="n">
-        <v>0.8223518897338907</v>
+        <v>0.8219284801273209</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="C110" t="n">
-        <v>0.201717293092171</v>
+        <v>0.2024921961666338</v>
       </c>
       <c r="D110" t="n">
-        <v>0.8223531365230738</v>
+        <v>0.8217534309260184</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C111" t="n">
-        <v>0.2017172060720553</v>
+        <v>0.2024394226183862</v>
       </c>
       <c r="D111" t="n">
-        <v>0.8223538384192065</v>
+        <v>0.8217239974658226</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="C112" t="n">
-        <v>0.2017171548294739</v>
+        <v>0.2028215988237095</v>
       </c>
       <c r="D112" t="n">
-        <v>0.8223550205600616</v>
+        <v>0.8214971372473567</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="C113" t="n">
-        <v>0.2017171271524447</v>
+        <v>0.202444606656265</v>
       </c>
       <c r="D113" t="n">
-        <v>0.8223557686335713</v>
+        <v>0.8221906568038316</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="C114" t="n">
-        <v>0.2017171147520817</v>
+        <v>0.2023856245356315</v>
       </c>
       <c r="D114" t="n">
-        <v>0.8223560918752115</v>
+        <v>0.821500729847299</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="C115" t="n">
-        <v>0.2017171120216113</v>
+        <v>0.2023707590794961</v>
       </c>
       <c r="D115" t="n">
-        <v>0.8223574494900997</v>
+        <v>0.8220080622191024</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="C116" t="n">
-        <v>0.2017171151979822</v>
+        <v>0.2023399191221626</v>
       </c>
       <c r="D116" t="n">
-        <v>0.8223576619060345</v>
+        <v>0.8220430831419335</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="C117" t="n">
-        <v>0.2017171217775695</v>
+        <v>0.2026597618659597</v>
       </c>
       <c r="D117" t="n">
-        <v>0.8223573756062963</v>
+        <v>0.8215947562226532</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="C118" t="n">
-        <v>0.2017171301168222</v>
+        <v>0.2026241514525391</v>
       </c>
       <c r="D118" t="n">
-        <v>0.8223574494900996</v>
+        <v>0.8215925120021238</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="C119" t="n">
-        <v>0.2017171391561337</v>
+        <v>0.2024069418580958</v>
       </c>
       <c r="D119" t="n">
-        <v>0.8223577357898381</v>
+        <v>0.8220721564185876</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="C120" t="n">
-        <v>0.2017171482305762</v>
+        <v>0.202546931196469</v>
       </c>
       <c r="D120" t="n">
-        <v>0.8223572740160665</v>
+        <v>0.8212117795275167</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>37</v>
+        <v>58</v>
       </c>
       <c r="C121" t="n">
-        <v>0.2017171569397702</v>
+        <v>0.2024637134620905</v>
       </c>
       <c r="D121" t="n">
-        <v>0.8223574771965261</v>
+        <v>0.8221370910463367</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="C122" t="n">
-        <v>0.2017171650589018</v>
+        <v>0.2024729230510603</v>
       </c>
       <c r="D122" t="n">
-        <v>0.8223571077775088</v>
+        <v>0.8212908351971984</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>l2</t>
+          <t>l1</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="C123" t="n">
-        <v>0.2017171724779662</v>
+        <v>0.2024499408301669</v>
       </c>
       <c r="D123" t="n">
-        <v>0.8223568676551476</v>
+        <v>0.8216248823435063</v>
       </c>
     </row>
     <row r="124">
@@ -3161,669 +3161,1949 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C124" t="n">
-        <v>0.2017171791605236</v>
+        <v>0.6931471805599455</v>
       </c>
       <c r="D124" t="n">
-        <v>0.8223570616001316</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C125" t="n">
-        <v>0.6931471805599455</v>
+        <v>0.3906801576744426</v>
       </c>
       <c r="D125" t="n">
-        <v>0.5</v>
+        <v>0.8088056637919926</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C126" t="n">
-        <v>0.203429024337331</v>
+        <v>0.2545362417751943</v>
       </c>
       <c r="D126" t="n">
-        <v>0.8213042820494247</v>
+        <v>0.811068835517097</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C127" t="n">
-        <v>0.2033044983586932</v>
+        <v>0.210901485567246</v>
       </c>
       <c r="D127" t="n">
-        <v>0.8213886758239053</v>
+        <v>0.8145665686557994</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C128" t="n">
-        <v>0.2034473429671905</v>
+        <v>0.2064513030933844</v>
       </c>
       <c r="D128" t="n">
-        <v>0.8212465326215602</v>
+        <v>0.8174073639562058</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C129" t="n">
-        <v>0.2028761108005181</v>
+        <v>0.2040834515376947</v>
       </c>
       <c r="D129" t="n">
-        <v>0.8218403644562422</v>
+        <v>0.8196404649733098</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C130" t="n">
-        <v>0.2022788500204483</v>
+        <v>0.2029993016438274</v>
       </c>
       <c r="D130" t="n">
-        <v>0.8219411050222341</v>
+        <v>0.8208928785609141</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C131" t="n">
-        <v>0.2023560979265742</v>
+        <v>0.2024152001412173</v>
       </c>
       <c r="D131" t="n">
-        <v>0.8217317367942329</v>
+        <v>0.8215591257584437</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C132" t="n">
-        <v>0.2022824998393344</v>
+        <v>0.2021481215593203</v>
       </c>
       <c r="D132" t="n">
-        <v>0.821857237669853</v>
+        <v>0.8217782004711218</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C133" t="n">
-        <v>0.2027189285291956</v>
+        <v>0.2019847968926103</v>
       </c>
       <c r="D133" t="n">
-        <v>0.8222566996886324</v>
+        <v>0.8219988452146232</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C134" t="n">
-        <v>0.2025448747717562</v>
+        <v>0.2018962511558601</v>
       </c>
       <c r="D134" t="n">
-        <v>0.8214038681809879</v>
+        <v>0.8220793600894231</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C135" t="n">
-        <v>0.2025648907284537</v>
+        <v>0.2018349437256716</v>
       </c>
       <c r="D135" t="n">
-        <v>0.8215819096763299</v>
+        <v>0.8221670139867304</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C136" t="n">
-        <v>0.2022587919412188</v>
+        <v>0.2017970290297426</v>
       </c>
       <c r="D136" t="n">
-        <v>0.8219981894958676</v>
+        <v>0.8222180769303837</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C137" t="n">
-        <v>0.2023066257940584</v>
+        <v>0.2017706927938434</v>
       </c>
       <c r="D137" t="n">
-        <v>0.8217900403506234</v>
+        <v>0.8222581127163733</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C138" t="n">
-        <v>0.2029919206012917</v>
+        <v>0.2017534903193746</v>
       </c>
       <c r="D138" t="n">
-        <v>0.8218829122915489</v>
+        <v>0.822279280426059</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C139" t="n">
-        <v>0.2028638322599649</v>
+        <v>0.2017416439753799</v>
       </c>
       <c r="D139" t="n">
-        <v>0.8214052904442041</v>
+        <v>0.8223010022642707</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C140" t="n">
-        <v>0.2024673755477015</v>
+        <v>0.2017337112271332</v>
       </c>
       <c r="D140" t="n">
-        <v>0.8221516923329918</v>
+        <v>0.8223150771288262</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C141" t="n">
-        <v>0.2027794962639662</v>
+        <v>0.2017282807899307</v>
       </c>
       <c r="D141" t="n">
-        <v>0.8216779586208033</v>
+        <v>0.8223243033687809</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C142" t="n">
-        <v>0.2024307981990134</v>
+        <v>0.2017246082583725</v>
       </c>
       <c r="D142" t="n">
-        <v>0.8220603904228896</v>
+        <v>0.8223317379265023</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C143" t="n">
-        <v>0.2026610839883875</v>
+        <v>0.2017221083889447</v>
       </c>
       <c r="D143" t="n">
-        <v>0.8215797762815056</v>
+        <v>0.8223356907099862</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C144" t="n">
-        <v>0.2024124223497717</v>
+        <v>0.2017204173772831</v>
       </c>
       <c r="D144" t="n">
-        <v>0.8216567262627894</v>
+        <v>0.8223408441052764</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C145" t="n">
-        <v>0.2025045778434697</v>
+        <v>0.201719273840277</v>
       </c>
       <c r="D145" t="n">
-        <v>0.8211229896667314</v>
+        <v>0.8223436701607579</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C146" t="n">
-        <v>0.2027715999108548</v>
+        <v>0.201718505792623</v>
       </c>
       <c r="D146" t="n">
-        <v>0.8216031974471965</v>
+        <v>0.8223464500388623</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C147" t="n">
-        <v>0.2024472117495033</v>
+        <v>0.2017179930012444</v>
       </c>
       <c r="D147" t="n">
-        <v>0.8217539204062161</v>
+        <v>0.822348823556048</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C148" t="n">
-        <v>0.2023473287687466</v>
+        <v>0.2017176543508925</v>
       </c>
       <c r="D148" t="n">
-        <v>0.8218611442759599</v>
+        <v>0.8223504674706743</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C149" t="n">
-        <v>0.2029077491013788</v>
+        <v>0.2017174337751697</v>
       </c>
       <c r="D149" t="n">
-        <v>0.8206190097725091</v>
+        <v>0.8223518897338907</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C150" t="n">
-        <v>0.2022474621488154</v>
+        <v>0.201717293092171</v>
       </c>
       <c r="D150" t="n">
-        <v>0.8222081765007225</v>
+        <v>0.8223531365230738</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C151" t="n">
-        <v>0.202805069611872</v>
+        <v>0.2017172060720553</v>
       </c>
       <c r="D151" t="n">
-        <v>0.8214714533901855</v>
+        <v>0.8223538384192065</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C152" t="n">
-        <v>0.2024076537133151</v>
+        <v>0.2017171548294739</v>
       </c>
       <c r="D152" t="n">
-        <v>0.8215984411773498</v>
+        <v>0.8223550205600616</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C153" t="n">
-        <v>0.2028990700927421</v>
+        <v>0.2017171271524447</v>
       </c>
       <c r="D153" t="n">
-        <v>0.8215335711979286</v>
+        <v>0.8223557686335713</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C154" t="n">
-        <v>0.2024048717586452</v>
+        <v>0.2017171147520817</v>
       </c>
       <c r="D154" t="n">
-        <v>0.822253014733936</v>
+        <v>0.8223560918752115</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C155" t="n">
-        <v>0.2024417669294848</v>
+        <v>0.2017171120216113</v>
       </c>
       <c r="D155" t="n">
-        <v>0.8219478192128716</v>
+        <v>0.8223574494900997</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C156" t="n">
-        <v>0.2025264713791506</v>
+        <v>0.2017171151979822</v>
       </c>
       <c r="D156" t="n">
-        <v>0.822029479286625</v>
+        <v>0.8223576619060345</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C157" t="n">
-        <v>0.2025280258441192</v>
+        <v>0.2017171217775695</v>
       </c>
       <c r="D157" t="n">
-        <v>0.8215229873430857</v>
+        <v>0.8223573756062963</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C158" t="n">
-        <v>0.2029414581403012</v>
+        <v>0.2017171301168222</v>
       </c>
       <c r="D158" t="n">
-        <v>0.8216330649747374</v>
+        <v>0.8223574494900996</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C159" t="n">
-        <v>0.2022000488381064</v>
+        <v>0.2017171391561337</v>
       </c>
       <c r="D159" t="n">
-        <v>0.8221653700721039</v>
+        <v>0.8223577357898381</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C160" t="n">
-        <v>0.2025579029535388</v>
+        <v>0.2017171482305762</v>
       </c>
       <c r="D160" t="n">
-        <v>0.8214163083663922</v>
+        <v>0.8223572740160665</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C161" t="n">
-        <v>0.2028471225536733</v>
+        <v>0.2017171569397702</v>
       </c>
       <c r="D161" t="n">
-        <v>0.8212976232716397</v>
+        <v>0.8223574771965261</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C162" t="n">
-        <v>0.2024558302600974</v>
+        <v>0.2017171650589018</v>
       </c>
       <c r="D162" t="n">
-        <v>0.8218800954715425</v>
+        <v>0.8223571077775088</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C163" t="n">
-        <v>0.2024902052793535</v>
+        <v>0.2017171724779662</v>
       </c>
       <c r="D163" t="n">
-        <v>0.8215956243573437</v>
+        <v>0.8223568676551476</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>elasticnet</t>
+          <t>l2</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C164" t="n">
-        <v>0.202916896304119</v>
+        <v>0.2017171791605236</v>
       </c>
       <c r="D164" t="n">
-        <v>0.8213447980801368</v>
+        <v>0.8223570616001316</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>41</v>
+      </c>
+      <c r="C165" t="n">
+        <v>0.2017171851158532</v>
+      </c>
+      <c r="D165" t="n">
+        <v>0.8223570985420332</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>42</v>
+      </c>
+      <c r="C166" t="n">
+        <v>0.2017171903803184</v>
+      </c>
+      <c r="D166" t="n">
+        <v>0.8223569138325247</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>43</v>
+      </c>
+      <c r="C167" t="n">
+        <v>0.201717195005035</v>
+      </c>
+      <c r="D167" t="n">
+        <v>0.822356876890623</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>44</v>
+      </c>
+      <c r="C168" t="n">
+        <v>0.2017171990478408</v>
+      </c>
+      <c r="D168" t="n">
+        <v>0.8223570431291808</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>45</v>
+      </c>
+      <c r="C169" t="n">
+        <v>0.2017172025681844</v>
+      </c>
+      <c r="D169" t="n">
+        <v>0.8223570893065579</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>46</v>
+      </c>
+      <c r="C170" t="n">
+        <v>0.2017172056239827</v>
+      </c>
+      <c r="D170" t="n">
+        <v>0.8223571262484597</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>47</v>
+      </c>
+      <c r="C171" t="n">
+        <v>0.2017172082697929</v>
+      </c>
+      <c r="D171" t="n">
+        <v>0.8223571170129841</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>48</v>
+      </c>
+      <c r="C172" t="n">
+        <v>0.201717210555852</v>
+      </c>
+      <c r="D172" t="n">
+        <v>0.8223569507744265</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>49</v>
+      </c>
+      <c r="C173" t="n">
+        <v>0.201717212527679</v>
+      </c>
+      <c r="D173" t="n">
+        <v>0.822356960009902</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>50</v>
+      </c>
+      <c r="C174" t="n">
+        <v>0.2017172142260321</v>
+      </c>
+      <c r="D174" t="n">
+        <v>0.8223570431291808</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>51</v>
+      </c>
+      <c r="C175" t="n">
+        <v>0.2017172156870821</v>
+      </c>
+      <c r="D175" t="n">
+        <v>0.822357135483935</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>52</v>
+      </c>
+      <c r="C176" t="n">
+        <v>0.2017172169427091</v>
+      </c>
+      <c r="D176" t="n">
+        <v>0.8223571077775088</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>53</v>
+      </c>
+      <c r="C177" t="n">
+        <v>0.2017172180208604</v>
+      </c>
+      <c r="D177" t="n">
+        <v>0.8223569784808528</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>54</v>
+      </c>
+      <c r="C178" t="n">
+        <v>0.2017172189459318</v>
+      </c>
+      <c r="D178" t="n">
+        <v>0.8223569323034756</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>55</v>
+      </c>
+      <c r="C179" t="n">
+        <v>0.2017172197391459</v>
+      </c>
+      <c r="D179" t="n">
+        <v>0.8223569969518036</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>56</v>
+      </c>
+      <c r="C180" t="n">
+        <v>0.201717220418914</v>
+      </c>
+      <c r="D180" t="n">
+        <v>0.8223570061872791</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>57</v>
+      </c>
+      <c r="C181" t="n">
+        <v>0.2017172210011722</v>
+      </c>
+      <c r="D181" t="n">
+        <v>0.8223570893065579</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>58</v>
+      </c>
+      <c r="C182" t="n">
+        <v>0.2017172214996883</v>
+      </c>
+      <c r="D182" t="n">
+        <v>0.8223571262484596</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>59</v>
+      </c>
+      <c r="C183" t="n">
+        <v>0.2017172219263381</v>
+      </c>
+      <c r="D183" t="n">
+        <v>0.8223570985420332</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>60</v>
+      </c>
+      <c r="C184" t="n">
+        <v>0.2017172222913524</v>
+      </c>
+      <c r="D184" t="n">
+        <v>0.8223570708356071</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
           <t>elasticnet</t>
         </is>
       </c>
-      <c r="B165" t="n">
+      <c r="B185" t="n">
+        <v>0</v>
+      </c>
+      <c r="C185" t="n">
+        <v>0.6931471805599455</v>
+      </c>
+      <c r="D185" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>1</v>
+      </c>
+      <c r="C186" t="n">
+        <v>0.203376296386073</v>
+      </c>
+      <c r="D186" t="n">
+        <v>0.8219267161515138</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>2</v>
+      </c>
+      <c r="C187" t="n">
+        <v>0.2027042655026061</v>
+      </c>
+      <c r="D187" t="n">
+        <v>0.8216868062062653</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>3</v>
+      </c>
+      <c r="C188" t="n">
+        <v>0.2024086736907048</v>
+      </c>
+      <c r="D188" t="n">
+        <v>0.8219236222672448</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>4</v>
+      </c>
+      <c r="C189" t="n">
+        <v>0.2027390017382703</v>
+      </c>
+      <c r="D189" t="n">
+        <v>0.821259111339096</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>5</v>
+      </c>
+      <c r="C190" t="n">
+        <v>0.2025934316318969</v>
+      </c>
+      <c r="D190" t="n">
+        <v>0.8219132785347629</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>6</v>
+      </c>
+      <c r="C191" t="n">
+        <v>0.2025183657019638</v>
+      </c>
+      <c r="D191" t="n">
+        <v>0.8218167308746164</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>7</v>
+      </c>
+      <c r="C192" t="n">
+        <v>0.2027857996512158</v>
+      </c>
+      <c r="D192" t="n">
+        <v>0.8214336156473483</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>8</v>
+      </c>
+      <c r="C193" t="n">
+        <v>0.2026281033351193</v>
+      </c>
+      <c r="D193" t="n">
+        <v>0.8209429163667945</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>9</v>
+      </c>
+      <c r="C194" t="n">
+        <v>0.2025026206305377</v>
+      </c>
+      <c r="D194" t="n">
+        <v>0.8213014929358449</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>10</v>
+      </c>
+      <c r="C195" t="n">
+        <v>0.2026044835485934</v>
+      </c>
+      <c r="D195" t="n">
+        <v>0.8215241233065638</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>11</v>
+      </c>
+      <c r="C196" t="n">
+        <v>0.202522256591297</v>
+      </c>
+      <c r="D196" t="n">
+        <v>0.8220994010711065</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>12</v>
+      </c>
+      <c r="C197" t="n">
+        <v>0.2026856673355794</v>
+      </c>
+      <c r="D197" t="n">
+        <v>0.8212448794714581</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>13</v>
+      </c>
+      <c r="C198" t="n">
+        <v>0.2028489376670972</v>
+      </c>
+      <c r="D198" t="n">
+        <v>0.8209733564938124</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>14</v>
+      </c>
+      <c r="C199" t="n">
+        <v>0.2024604923349713</v>
+      </c>
+      <c r="D199" t="n">
+        <v>0.8221181490862296</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>15</v>
+      </c>
+      <c r="C200" t="n">
+        <v>0.2022229089851154</v>
+      </c>
+      <c r="D200" t="n">
+        <v>0.8218327636599633</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>16</v>
+      </c>
+      <c r="C201" t="n">
+        <v>0.2022562194419317</v>
+      </c>
+      <c r="D201" t="n">
+        <v>0.8218973288686953</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>17</v>
+      </c>
+      <c r="C202" t="n">
+        <v>0.2024794269043794</v>
+      </c>
+      <c r="D202" t="n">
+        <v>0.8214284530165828</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>18</v>
+      </c>
+      <c r="C203" t="n">
+        <v>0.2024067434807453</v>
+      </c>
+      <c r="D203" t="n">
+        <v>0.8215038514379945</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>19</v>
+      </c>
+      <c r="C204" t="n">
+        <v>0.2024664267306339</v>
+      </c>
+      <c r="D204" t="n">
+        <v>0.8214674451938488</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>20</v>
+      </c>
+      <c r="C205" t="n">
+        <v>0.2027214253971167</v>
+      </c>
+      <c r="D205" t="n">
+        <v>0.8214765051952458</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>21</v>
+      </c>
+      <c r="C206" t="n">
+        <v>0.2027763365151587</v>
+      </c>
+      <c r="D206" t="n">
+        <v>0.821583738300465</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>22</v>
+      </c>
+      <c r="C207" t="n">
+        <v>0.202469074810788</v>
+      </c>
+      <c r="D207" t="n">
+        <v>0.8209176665769687</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>23</v>
+      </c>
+      <c r="C208" t="n">
+        <v>0.2027974822155681</v>
+      </c>
+      <c r="D208" t="n">
+        <v>0.8214533610938179</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>24</v>
+      </c>
+      <c r="C209" t="n">
+        <v>0.2024403378229874</v>
+      </c>
+      <c r="D209" t="n">
+        <v>0.8216393820399316</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>25</v>
+      </c>
+      <c r="C210" t="n">
+        <v>0.2024064722639387</v>
+      </c>
+      <c r="D210" t="n">
+        <v>0.821421905064503</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>26</v>
+      </c>
+      <c r="C211" t="n">
+        <v>0.2026350930388948</v>
+      </c>
+      <c r="D211" t="n">
+        <v>0.8221777640801311</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>27</v>
+      </c>
+      <c r="C212" t="n">
+        <v>0.202632895801049</v>
+      </c>
+      <c r="D212" t="n">
+        <v>0.8215622473491393</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>28</v>
+      </c>
+      <c r="C213" t="n">
+        <v>0.2022321538880047</v>
+      </c>
+      <c r="D213" t="n">
+        <v>0.8219863773227926</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>29</v>
+      </c>
+      <c r="C214" t="n">
+        <v>0.202274253715092</v>
+      </c>
+      <c r="D214" t="n">
+        <v>0.8219987528598689</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>30</v>
+      </c>
+      <c r="C215" t="n">
+        <v>0.2025233420351641</v>
+      </c>
+      <c r="D215" t="n">
+        <v>0.8214379655562759</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>31</v>
+      </c>
+      <c r="C216" t="n">
+        <v>0.2026449051789233</v>
+      </c>
+      <c r="D216" t="n">
+        <v>0.821595458118786</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>32</v>
+      </c>
+      <c r="C217" t="n">
+        <v>0.2025142369280395</v>
+      </c>
+      <c r="D217" t="n">
+        <v>0.8223135717463312</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>33</v>
+      </c>
+      <c r="C218" t="n">
+        <v>0.2024224357245681</v>
+      </c>
+      <c r="D218" t="n">
+        <v>0.8221288437667778</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>34</v>
+      </c>
+      <c r="C219" t="n">
+        <v>0.2028851922902798</v>
+      </c>
+      <c r="D219" t="n">
+        <v>0.8210054220645059</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>35</v>
+      </c>
+      <c r="C220" t="n">
+        <v>0.2027943414280469</v>
+      </c>
+      <c r="D220" t="n">
+        <v>0.8219159383516869</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>36</v>
+      </c>
+      <c r="C221" t="n">
+        <v>0.2024460796901385</v>
+      </c>
+      <c r="D221" t="n">
+        <v>0.8217222057835891</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>37</v>
+      </c>
+      <c r="C222" t="n">
+        <v>0.2029390416347083</v>
+      </c>
+      <c r="D222" t="n">
+        <v>0.820461323265015</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>38</v>
+      </c>
+      <c r="C223" t="n">
+        <v>0.202656244529427</v>
+      </c>
+      <c r="D223" t="n">
+        <v>0.8211525708945341</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>39</v>
+      </c>
+      <c r="C224" t="n">
+        <v>0.2026416842701361</v>
+      </c>
+      <c r="D224" t="n">
+        <v>0.8208698175787651</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
         <v>40</v>
       </c>
-      <c r="C165" t="n">
-        <v>0.2026972858690364</v>
-      </c>
-      <c r="D165" t="n">
-        <v>0.8212764740329047</v>
+      <c r="C225" t="n">
+        <v>0.2030174648600079</v>
+      </c>
+      <c r="D225" t="n">
+        <v>0.8211047218963304</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>41</v>
+      </c>
+      <c r="C226" t="n">
+        <v>0.2026564150890884</v>
+      </c>
+      <c r="D226" t="n">
+        <v>0.8216144739626966</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>42</v>
+      </c>
+      <c r="C227" t="n">
+        <v>0.2026195904165935</v>
+      </c>
+      <c r="D227" t="n">
+        <v>0.8218437631112004</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>43</v>
+      </c>
+      <c r="C228" t="n">
+        <v>0.2025515392104202</v>
+      </c>
+      <c r="D228" t="n">
+        <v>0.821297115320491</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>44</v>
+      </c>
+      <c r="C229" t="n">
+        <v>0.2021170730711528</v>
+      </c>
+      <c r="D229" t="n">
+        <v>0.8217798813276501</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>45</v>
+      </c>
+      <c r="C230" t="n">
+        <v>0.2026875062222676</v>
+      </c>
+      <c r="D230" t="n">
+        <v>0.8215127174944074</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>46</v>
+      </c>
+      <c r="C231" t="n">
+        <v>0.2027894699555995</v>
+      </c>
+      <c r="D231" t="n">
+        <v>0.8218987418964361</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>47</v>
+      </c>
+      <c r="C232" t="n">
+        <v>0.2022041626243121</v>
+      </c>
+      <c r="D232" t="n">
+        <v>0.8222969571260322</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>48</v>
+      </c>
+      <c r="C233" t="n">
+        <v>0.2024427526245237</v>
+      </c>
+      <c r="D233" t="n">
+        <v>0.8208481142115042</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>49</v>
+      </c>
+      <c r="C234" t="n">
+        <v>0.2022684472428646</v>
+      </c>
+      <c r="D234" t="n">
+        <v>0.8217371118409332</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>50</v>
+      </c>
+      <c r="C235" t="n">
+        <v>0.2022738624159174</v>
+      </c>
+      <c r="D235" t="n">
+        <v>0.8219054006742212</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>51</v>
+      </c>
+      <c r="C236" t="n">
+        <v>0.2026549889893333</v>
+      </c>
+      <c r="D236" t="n">
+        <v>0.8216393266270791</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>52</v>
+      </c>
+      <c r="C237" t="n">
+        <v>0.2025171153004346</v>
+      </c>
+      <c r="D237" t="n">
+        <v>0.8221702833450328</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>53</v>
+      </c>
+      <c r="C238" t="n">
+        <v>0.2023833630473995</v>
+      </c>
+      <c r="D238" t="n">
+        <v>0.8222254468397769</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>54</v>
+      </c>
+      <c r="C239" t="n">
+        <v>0.2023845895323994</v>
+      </c>
+      <c r="D239" t="n">
+        <v>0.8222370281259663</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>55</v>
+      </c>
+      <c r="C240" t="n">
+        <v>0.2023038407613106</v>
+      </c>
+      <c r="D240" t="n">
+        <v>0.8220577675478674</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>56</v>
+      </c>
+      <c r="C241" t="n">
+        <v>0.2022709768999565</v>
+      </c>
+      <c r="D241" t="n">
+        <v>0.8217181144679735</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>57</v>
+      </c>
+      <c r="C242" t="n">
+        <v>0.2028137879999375</v>
+      </c>
+      <c r="D242" t="n">
+        <v>0.8211155643444856</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>58</v>
+      </c>
+      <c r="C243" t="n">
+        <v>0.2023865600514186</v>
+      </c>
+      <c r="D243" t="n">
+        <v>0.8215320842863845</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>59</v>
+      </c>
+      <c r="C244" t="n">
+        <v>0.2021880727735407</v>
+      </c>
+      <c r="D244" t="n">
+        <v>0.8218113096505389</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>elasticnet</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>60</v>
+      </c>
+      <c r="C245" t="n">
+        <v>0.202498287458618</v>
+      </c>
+      <c r="D245" t="n">
+        <v>0.8220759152570876</v>
       </c>
     </row>
   </sheetData>
@@ -3837,7 +5117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3863,30 +5143,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>TotalSeconds</t>
+          <t>RecalDelta</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>RecalDelta</t>
+          <t>RecalLogLoss</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>FinalLogLoss</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>FinalAUROC</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>RecalLogLoss</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>RecalAUROC</t>
         </is>
@@ -3902,28 +5167,19 @@
         <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>1.119</v>
+        <v>1.6213</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0049</v>
+        <v>0.0046</v>
       </c>
       <c r="E2" t="n">
-        <v>1.123</v>
+        <v>0.004912898904571858</v>
       </c>
       <c r="F2" t="n">
-        <v>0.004798500043224268</v>
+        <v>0.2017165594625326</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2017171779479682</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.8223570800710825</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.2017165466116977</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.8223570800710825</v>
+        <v>0.8223570616001317</v>
       </c>
     </row>
     <row r="3">
@@ -3933,31 +5189,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C3" t="n">
-        <v>1.259</v>
+        <v>1.6936</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0069</v>
+        <v>0.0059</v>
       </c>
       <c r="E3" t="n">
-        <v>1.266</v>
+        <v>0.1070837433996043</v>
       </c>
       <c r="F3" t="n">
-        <v>0.07076937857726544</v>
+        <v>0.2021469260941534</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2024485277561125</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.8215813832542304</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.2023167026472674</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.8215813832542304</v>
+        <v>0.8216248823435063</v>
       </c>
     </row>
     <row r="4">
@@ -3970,28 +5217,19 @@
         <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>1.232</v>
+        <v>1.6578</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0045</v>
+        <v>0.0046</v>
       </c>
       <c r="E4" t="n">
-        <v>1.237</v>
+        <v>0.004913019321012238</v>
       </c>
       <c r="F4" t="n">
-        <v>0.00479863490695206</v>
+        <v>0.2017165605081437</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2017171791605236</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.8223570616001316</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.2017165477877157</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.8223570616001316</v>
+        <v>0.8223570708356071</v>
       </c>
     </row>
     <row r="5">
@@ -4001,31 +5239,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C5" t="n">
-        <v>1.328</v>
+        <v>1.706</v>
       </c>
       <c r="D5" t="n">
-        <v>0.006</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>1.334</v>
+        <v>0.09788354899420276</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1219667429884901</v>
+        <v>0.2022490841581845</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2026972858690364</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.8212764740329047</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.2023084817093646</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.8212764740329047</v>
+        <v>0.8220759152570876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>